<commit_message>
georganiseerd in happen + screenshots toegevoegd
</commit_message>
<xml_diff>
--- a/Logboeken/Logboek Eddie.xlsx
+++ b/Logboeken/Logboek Eddie.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="22202"/>
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="22220"/>
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="-440" windowWidth="33600" windowHeight="21000" tabRatio="500"/>
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="20">
   <si>
     <t>Datum</t>
   </si>
@@ -61,6 +61,24 @@
   </si>
   <si>
     <t>Titanium Studio leren</t>
+  </si>
+  <si>
+    <t>Voorbereiding voor gesprek met opdrachtgever maken</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rapport maken voor de presentatie </t>
+  </si>
+  <si>
+    <t>1,5 uur</t>
+  </si>
+  <si>
+    <t>Gesprek met opdrachtgever</t>
+  </si>
+  <si>
+    <t>Presentatie van ons rapport</t>
+  </si>
+  <si>
+    <t>Begin gemaakt met de app: De kaart</t>
   </si>
 </sst>
 </file>
@@ -124,10 +142,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normaal" xfId="0" builtinId="0"/>
@@ -467,8 +485,8 @@
     <col min="3" max="3" width="13.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" s="5" customFormat="1" ht="45">
-      <c r="A1" s="5" t="s">
+    <row r="1" spans="1:3" s="6" customFormat="1" ht="45">
+      <c r="A1" s="6" t="s">
         <v>6</v>
       </c>
     </row>
@@ -479,7 +497,7 @@
       <c r="B2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="C2" s="5" t="s">
         <v>7</v>
       </c>
     </row>
@@ -575,30 +593,72 @@
       <c r="A11" s="3">
         <v>41023</v>
       </c>
-      <c r="B11" s="4"/>
+      <c r="B11" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C11" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="12" spans="1:3">
-      <c r="A12" s="4"/>
-      <c r="B12" s="4"/>
+      <c r="A12" s="3">
+        <v>41024</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C12" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="13" spans="1:3">
-      <c r="A13" s="4"/>
-      <c r="B13" s="4"/>
+      <c r="A13" s="3">
+        <v>41024</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C13" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="14" spans="1:3">
-      <c r="A14" s="4"/>
-      <c r="B14" s="4"/>
+      <c r="A14" s="3">
+        <v>41025</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C14" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="15" spans="1:3">
-      <c r="A15" s="4"/>
-      <c r="B15" s="4"/>
+      <c r="A15" s="3">
+        <v>41025</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C15" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="16" spans="1:3">
-      <c r="A16" s="4"/>
-      <c r="B16" s="4"/>
+      <c r="A16" s="3">
+        <v>41026</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="C16" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="17" spans="1:2">
-      <c r="A17" s="4"/>
+      <c r="A17" s="3">
+        <v>41035</v>
+      </c>
       <c r="B17" s="4"/>
     </row>
     <row r="18" spans="1:2">

</xml_diff>

<commit_message>
logboeken + notulen en deelrapport gemaakt
</commit_message>
<xml_diff>
--- a/Logboeken/Logboek Eddie.xlsx
+++ b/Logboeken/Logboek Eddie.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="39">
   <si>
     <t>Datum</t>
   </si>
@@ -121,6 +121,21 @@
   </si>
   <si>
     <t>Verder gewerkt aan het rapport</t>
+  </si>
+  <si>
+    <t>Bugs fixen</t>
+  </si>
+  <si>
+    <t>4,5 uur</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Deelrapport gemaakt </t>
+  </si>
+  <si>
+    <t>Searchbar op de map verwijderd + settings voor iPhone verbeterd</t>
+  </si>
+  <si>
+    <t>2 uur</t>
   </si>
 </sst>
 </file>
@@ -873,67 +888,95 @@
         <v>25</v>
       </c>
     </row>
-    <row r="33" spans="1:2">
-      <c r="A33" s="4"/>
-      <c r="B33" s="4"/>
-    </row>
-    <row r="34" spans="1:2">
-      <c r="A34" s="4"/>
-      <c r="B34" s="4"/>
-    </row>
-    <row r="35" spans="1:2">
-      <c r="A35" s="4"/>
-      <c r="B35" s="4"/>
-    </row>
-    <row r="36" spans="1:2">
-      <c r="A36" s="4"/>
-      <c r="B36" s="4"/>
-    </row>
-    <row r="37" spans="1:2">
+    <row r="33" spans="1:3">
+      <c r="A33" s="3">
+        <v>41053</v>
+      </c>
+      <c r="B33" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="C33" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3">
+      <c r="A34" s="3">
+        <v>41054</v>
+      </c>
+      <c r="B34" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="C34" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3">
+      <c r="A35" s="3">
+        <v>41058</v>
+      </c>
+      <c r="B35" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="C35" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3">
+      <c r="A36" s="3">
+        <v>41058</v>
+      </c>
+      <c r="B36" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="C36" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3">
       <c r="A37" s="4"/>
       <c r="B37" s="4"/>
     </row>
-    <row r="38" spans="1:2">
+    <row r="38" spans="1:3">
       <c r="A38" s="4"/>
       <c r="B38" s="4"/>
     </row>
-    <row r="39" spans="1:2">
+    <row r="39" spans="1:3">
       <c r="A39" s="4"/>
       <c r="B39" s="4"/>
     </row>
-    <row r="40" spans="1:2">
+    <row r="40" spans="1:3">
       <c r="A40" s="4"/>
       <c r="B40" s="4"/>
     </row>
-    <row r="41" spans="1:2">
+    <row r="41" spans="1:3">
       <c r="A41" s="4"/>
       <c r="B41" s="4"/>
     </row>
-    <row r="42" spans="1:2">
+    <row r="42" spans="1:3">
       <c r="A42" s="4"/>
       <c r="B42" s="4"/>
     </row>
-    <row r="43" spans="1:2">
+    <row r="43" spans="1:3">
       <c r="A43" s="4"/>
       <c r="B43" s="4"/>
     </row>
-    <row r="44" spans="1:2">
+    <row r="44" spans="1:3">
       <c r="A44" s="4"/>
       <c r="B44" s="4"/>
     </row>
-    <row r="45" spans="1:2">
+    <row r="45" spans="1:3">
       <c r="A45" s="4"/>
       <c r="B45" s="4"/>
     </row>
-    <row r="46" spans="1:2">
+    <row r="46" spans="1:3">
       <c r="A46" s="4"/>
       <c r="B46" s="4"/>
     </row>
-    <row r="47" spans="1:2">
+    <row r="47" spans="1:3">
       <c r="A47" s="4"/>
       <c r="B47" s="4"/>
     </row>
-    <row r="48" spans="1:2">
+    <row r="48" spans="1:3">
       <c r="A48" s="4"/>
       <c r="B48" s="4"/>
     </row>

</xml_diff>

<commit_message>
logboeken bijgewerkt + rapport screenshot
</commit_message>
<xml_diff>
--- a/Logboeken/Logboek Eddie.xlsx
+++ b/Logboeken/Logboek Eddie.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="22221"/>
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
   <bookViews>
-    <workbookView xWindow="5240" yWindow="2780" windowWidth="25600" windowHeight="16060" tabRatio="500"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="33600" windowHeight="18580" tabRatio="500"/>
   </bookViews>
   <sheets>
     <sheet name="Blad1" sheetId="1" r:id="rId1"/>
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="45">
   <si>
     <t>Datum</t>
   </si>
@@ -148,6 +148,12 @@
   </si>
   <si>
     <t>Het Rapport optimaliseren</t>
+  </si>
+  <si>
+    <t>Apps klaargemaakt voor gesprek met Opdrachtgever</t>
+  </si>
+  <si>
+    <t>Rapport volledig gemaakt</t>
   </si>
 </sst>
 </file>
@@ -996,18 +1002,39 @@
       <c r="B41" s="4" t="s">
         <v>42</v>
       </c>
+      <c r="C41" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="42" spans="1:3">
-      <c r="A42" s="4"/>
-      <c r="B42" s="4"/>
+      <c r="A42" s="3">
+        <v>41066</v>
+      </c>
+      <c r="B42" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="C42" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="43" spans="1:3">
-      <c r="A43" s="4"/>
-      <c r="B43" s="4"/>
+      <c r="A43" s="3">
+        <v>41067</v>
+      </c>
+      <c r="B43" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="C43" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="44" spans="1:3">
-      <c r="A44" s="4"/>
-      <c r="B44" s="4"/>
+      <c r="A44" s="3">
+        <v>41071</v>
+      </c>
+      <c r="B44" s="4" t="s">
+        <v>44</v>
+      </c>
     </row>
     <row r="45" spans="1:3">
       <c r="A45" s="4"/>

</xml_diff>